<commit_message>
Changed to Mapser and updated some DTOS
</commit_message>
<xml_diff>
--- a/LoyaltyCRM.Tests/TestData/ImportSample.xlsx
+++ b/LoyaltyCRM.Tests/TestData/ImportSample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SPAC-O-5\Visual Studio Projects\LoyaltyCRM\LoyaltyCRM.Tests\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7C3096E-6B8D-4991-A7A0-2CD4DD102D8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30D08391-73BB-4389-AD8C-4089CC37E198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="41">
   <si>
     <t>Kortnummer</t>
   </si>
@@ -153,6 +153,9 @@
   </si>
   <si>
     <t>InvalidPhone</t>
+  </si>
+  <si>
+    <t>+45-12345667</t>
   </si>
 </sst>
 </file>
@@ -206,11 +209,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -548,7 +552,7 @@
       <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D2" t="s">
@@ -565,8 +569,8 @@
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
-        <v>6</v>
+      <c r="C3" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="D3" t="s">
         <v>10</v>
@@ -582,7 +586,7 @@
       <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D4" t="s">

</xml_diff>